<commit_message>
feat : anomalies introduites sur toutes les tables
</commit_message>
<xml_diff>
--- a/data/raw/corrections_metier_articles.xlsx
+++ b/data/raw/corrections_metier_articles.xlsx
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ART064</t>
+          <t>ART061</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -451,22 +451,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Haute</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ART001</t>
+          <t>ART065</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BETON</t>
+          <t>ARMATURE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -475,13 +475,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ART071</t>
+          <t>ART040</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -491,11 +491,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Haute</t>
+          <t>Moyenne</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5">
@@ -506,27 +506,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BETON</t>
+          <t>ISOLATION</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Haute</t>
+          <t>Basse</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ART060</t>
+          <t>ART086</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BETON</t>
+          <t>ARMATURE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -535,103 +535,103 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ART084</t>
+          <t>ART020</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>BETON</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Basse</t>
+          <t>Haute</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ART048</t>
+          <t>ART013</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>BETON</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Haute</t>
+          <t>Basse</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ART041</t>
+          <t>ART011</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ISOLATION</t>
+          <t>BETON</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Basse</t>
+          <t>Moyenne</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ART084</t>
+          <t>ART053</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>ISOLATION</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Basse</t>
+          <t>Haute</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ART008</t>
+          <t>ART043</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ISOLATION</t>
+          <t>BETON</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Basse</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -641,52 +641,52 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ART098</t>
+          <t>ART046</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ISOLATION</t>
+          <t>ARMATURE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Basse</t>
+          <t>Haute</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>80</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ART081</t>
+          <t>ART076</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>BETON</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Basse</t>
+          <t>Moyenne</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ART087</t>
+          <t>ART093</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>ISOLATION</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -701,12 +701,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ART096</t>
+          <t>ART088</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>ISOLATION</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -721,7 +721,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ART004</t>
+          <t>ART017</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Basse</t>
+          <t>Moyenne</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ART072</t>
+          <t>ART006</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -751,17 +751,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Haute</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ART055</t>
+          <t>ART023</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -775,13 +775,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ART092</t>
+          <t>ART097</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -791,37 +791,37 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Haute</t>
+          <t>Basse</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ART051</t>
+          <t>ART025</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>ISOLATION</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Basse</t>
+          <t>Moyenne</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ART058</t>
+          <t>ART097</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -831,37 +831,37 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Haute</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>80</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ART093</t>
+          <t>ART087</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>BETON</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Basse</t>
+          <t>Haute</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ART045</t>
+          <t>ART006</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -871,37 +871,37 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Haute</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ART010</t>
+          <t>ART025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>ISOLATION</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Basse</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ART045</t>
+          <t>ART084</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -926,22 +926,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>ISOLATION</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Haute</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ART065</t>
+          <t>ART034</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -951,17 +951,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Haute</t>
+          <t>Moyenne</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ART060</t>
+          <t>ART078</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -975,13 +975,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ART087</t>
+          <t>ART050</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -991,37 +991,37 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Basse</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ART047</t>
+          <t>ART075</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ARMATURE</t>
+          <t>BETON</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Basse</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ART099</t>
+          <t>ART086</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1031,11 +1031,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Haute</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>